<commit_message>
fix: filter empty rows in Excel export to prevent ghost DC rows after last data
</commit_message>
<xml_diff>
--- a/template/Template_Solutions_NVN.xlsx
+++ b/template/Template_Solutions_NVN.xlsx
@@ -28,7 +28,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000F172A"/>
       <sz val="11"/>
     </font>
     <font>
@@ -39,7 +38,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="000F172A"/>
       <sz val="11"/>
     </font>
     <font>
@@ -63,13 +61,19 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="medium"/>
     </border>
     <border>
       <left style="thin">
@@ -97,13 +101,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>

</xml_diff>